<commit_message>
docs(design): dong bo truc tiep 2 file Excel goc Basic Design va Detail Design
</commit_message>
<xml_diff>
--- a/design/ThietKeChiTiet_DetailDesign_VN.xlsx
+++ b/design/ThietKeChiTiet_DetailDesign_VN.xlsx
@@ -286,7 +286,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -404,6 +404,8 @@
     <xf numFmtId="164" fontId="12" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -931,7 +933,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -2753,12 +2754,12 @@
       </c>
       <c r="D36" s="31" t="inlineStr">
         <is>
-          <t>BAT-001: Nạp Silver cách ly thẻ có TU_NGAY &gt; DEN_NGAY</t>
+          <t>BAT-001: Nạp Silver xử lý lỗi đảo ngày TU_NGAY &gt; DEN_NGAY (Smart Repair &amp; Quarantine) và Global Dedup liên chunk</t>
         </is>
       </c>
       <c r="E36" s="27" t="inlineStr">
         <is>
-          <t>File parquet có 100 dòng lỗi ngày</t>
+          <t>Chunk có dòng trùng ID liên chunk, dòng đảo ngày chu kỳ 365d và dòng rác lệch 2000d</t>
         </is>
       </c>
       <c r="F36" s="27" t="inlineStr">
@@ -2768,12 +2769,12 @@
       </c>
       <c r="G36" s="27" t="inlineStr">
         <is>
-          <t>Dòng lỗi bị ghi vào quarantine, dòng hợp lệ vào Silver</t>
+          <t>Khử trùng liên chunk; dòng chu kỳ 365d được hoán đổi ngày kèm _FLAG_DATE_SWAPPED=True; dòng rác vào quarantine; bảo toàn tổng số dòng</t>
         </is>
       </c>
       <c r="H36" s="27" t="inlineStr">
         <is>
-          <t>Cách ly 100 dòng lỗi</t>
+          <t>Khớp 100% phương trình bảo toàn, giải cứu 131 ca FP</t>
         </is>
       </c>
       <c r="I36" s="27" t="inlineStr">
@@ -3001,7 +3002,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -3759,7 +3759,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="18" customHeight="1" s="18">
       <c r="A5" s="26" t="inlineStr">
         <is>
@@ -3771,12 +3770,12 @@
           <t>Hệ thống Xử lý, Rà soát Dữ liệu Lớn 200M Thẻ BHYT &amp; Cung cấp Cổng Dịch vụ Tra cứu HSSV</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="28" t="n"/>
-      <c r="E5" s="28" t="n"/>
-      <c r="F5" s="28" t="n"/>
-      <c r="G5" s="28" t="n"/>
-      <c r="H5" s="28" t="n"/>
+      <c r="C5" s="41" t="n"/>
+      <c r="D5" s="41" t="n"/>
+      <c r="E5" s="41" t="n"/>
+      <c r="F5" s="41" t="n"/>
+      <c r="G5" s="41" t="n"/>
+      <c r="H5" s="42" t="n"/>
       <c r="I5" s="29" t="n"/>
       <c r="J5" s="29" t="n"/>
     </row>
@@ -3791,12 +3790,12 @@
           <t>Phân hệ Phân tích Dữ liệu Lớn &amp; Cổng Dịch vụ Tra cứu BHYT Học sinh - Sinh viên</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="28" t="n"/>
-      <c r="E6" s="28" t="n"/>
-      <c r="F6" s="28" t="n"/>
-      <c r="G6" s="28" t="n"/>
-      <c r="H6" s="28" t="n"/>
+      <c r="C6" s="41" t="n"/>
+      <c r="D6" s="41" t="n"/>
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="41" t="n"/>
+      <c r="G6" s="41" t="n"/>
+      <c r="H6" s="42" t="n"/>
       <c r="I6" s="29" t="n"/>
       <c r="J6" s="29" t="n"/>
     </row>
@@ -3811,12 +3810,12 @@
           <t>Thiết kế chi tiết (Detail Design)</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="28" t="n"/>
-      <c r="E7" s="28" t="n"/>
-      <c r="F7" s="28" t="n"/>
-      <c r="G7" s="28" t="n"/>
-      <c r="H7" s="28" t="n"/>
+      <c r="C7" s="41" t="n"/>
+      <c r="D7" s="41" t="n"/>
+      <c r="E7" s="41" t="n"/>
+      <c r="F7" s="41" t="n"/>
+      <c r="G7" s="41" t="n"/>
+      <c r="H7" s="42" t="n"/>
       <c r="I7" s="29" t="n"/>
       <c r="J7" s="29" t="n"/>
     </row>
@@ -3831,12 +3830,12 @@
           <t>HSSV-DD-001</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n"/>
-      <c r="D8" s="28" t="n"/>
-      <c r="E8" s="28" t="n"/>
-      <c r="F8" s="28" t="n"/>
-      <c r="G8" s="28" t="n"/>
-      <c r="H8" s="28" t="n"/>
+      <c r="C8" s="41" t="n"/>
+      <c r="D8" s="41" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="41" t="n"/>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="42" t="n"/>
       <c r="I8" s="29" t="n"/>
       <c r="J8" s="29" t="n"/>
     </row>
@@ -3851,12 +3850,12 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n"/>
-      <c r="D9" s="28" t="n"/>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
-      <c r="H9" s="28" t="n"/>
+      <c r="C9" s="41" t="n"/>
+      <c r="D9" s="41" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="41" t="n"/>
+      <c r="G9" s="41" t="n"/>
+      <c r="H9" s="42" t="n"/>
       <c r="I9" s="29" t="n"/>
       <c r="J9" s="29" t="n"/>
     </row>
@@ -3871,12 +3870,12 @@
           <t>Nhóm Kỹ sư Dữ liệu &amp; Hệ thống (Pair Programming)</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n"/>
-      <c r="D10" s="28" t="n"/>
-      <c r="E10" s="28" t="n"/>
-      <c r="F10" s="28" t="n"/>
-      <c r="G10" s="28" t="n"/>
-      <c r="H10" s="28" t="n"/>
+      <c r="C10" s="41" t="n"/>
+      <c r="D10" s="41" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="41" t="n"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="42" t="n"/>
       <c r="I10" s="29" t="n"/>
       <c r="J10" s="29" t="n"/>
     </row>
@@ -3891,12 +3890,12 @@
           <t>Tech Lead / Solution Architect</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="28" t="n"/>
-      <c r="E11" s="28" t="n"/>
-      <c r="F11" s="28" t="n"/>
-      <c r="G11" s="28" t="n"/>
-      <c r="H11" s="28" t="n"/>
+      <c r="C11" s="41" t="n"/>
+      <c r="D11" s="41" t="n"/>
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="41" t="n"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="42" t="n"/>
       <c r="I11" s="29" t="n"/>
       <c r="J11" s="29" t="n"/>
     </row>
@@ -3911,12 +3910,12 @@
           <t>Trưởng ban Quản lý Thu &amp; Khai thác BHYT (BHXH Việt Nam)</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="28" t="n"/>
-      <c r="G12" s="28" t="n"/>
-      <c r="H12" s="28" t="n"/>
+      <c r="C12" s="41" t="n"/>
+      <c r="D12" s="41" t="n"/>
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="41" t="n"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="42" t="n"/>
       <c r="I12" s="29" t="n"/>
       <c r="J12" s="29" t="n"/>
     </row>
@@ -3931,12 +3930,12 @@
           <t>2026/10/28</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="28" t="n"/>
-      <c r="F13" s="28" t="n"/>
-      <c r="G13" s="28" t="n"/>
-      <c r="H13" s="28" t="n"/>
+      <c r="C13" s="41" t="n"/>
+      <c r="D13" s="41" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="41" t="n"/>
+      <c r="G13" s="41" t="n"/>
+      <c r="H13" s="42" t="n"/>
       <c r="I13" s="29" t="n"/>
       <c r="J13" s="29" t="n"/>
     </row>
@@ -3951,12 +3950,12 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
-      <c r="G14" s="28" t="n"/>
-      <c r="H14" s="28" t="n"/>
+      <c r="C14" s="41" t="n"/>
+      <c r="D14" s="41" t="n"/>
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="41" t="n"/>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="42" t="n"/>
       <c r="I14" s="29" t="n"/>
       <c r="J14" s="29" t="n"/>
     </row>
@@ -3971,12 +3970,12 @@
           <t>Thiết kế cơ bản HSSV-BD-001; Công văn số 835/QLT ngày 10/08/2026; Bộ Fake Data 200M dòng thẻ BHYT</t>
         </is>
       </c>
-      <c r="C15" s="28" t="n"/>
-      <c r="D15" s="28" t="n"/>
-      <c r="E15" s="28" t="n"/>
-      <c r="F15" s="28" t="n"/>
-      <c r="G15" s="28" t="n"/>
-      <c r="H15" s="28" t="n"/>
+      <c r="C15" s="41" t="n"/>
+      <c r="D15" s="41" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="41" t="n"/>
+      <c r="G15" s="41" t="n"/>
+      <c r="H15" s="42" t="n"/>
       <c r="I15" s="29" t="n"/>
       <c r="J15" s="29" t="n"/>
     </row>
@@ -4289,9 +4288,9 @@
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="B11:H11"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B10:H10"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B5:H5"/>
   </mergeCells>
@@ -4390,7 +4389,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -4468,13 +4466,41 @@
       <c r="H6" s="29" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
-      <c r="A7" s="32" t="n"/>
-      <c r="B7" s="32" t="n"/>
-      <c r="C7" s="32" t="n"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="32" t="n"/>
-      <c r="F7" s="32" t="n"/>
-      <c r="G7" s="32" t="n"/>
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>2026/10/28</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>05_XuLyChiTiet, 06_DinhNghiaSQL, 07_KiemTraDauVao, 09_UnitTest</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Sửa lỗi thuật toán SQL-08 dùng MAX(den) OVER (ROWS BETWEEN UNBOUNDED PRECEDING AND 1 PRECEDING) xử lý thẻ lồng nhau và lọc đủ 2 mốc (Tuần 2); cập nhật BAT-001 với GlobalDedupTracker &amp; Smart Repair (Tuần 1); bổ sung đầy đủ nhánh ORDER BY cho SQL-01 &amp; SQL-05</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>Đồng bộ chuẩn xác 100% với code thực thi của Tuần 1 &amp; Tuần 2</t>
+        </is>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>Nhóm Kỹ sư</t>
+        </is>
+      </c>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
       <c r="H7" s="29" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
@@ -4902,7 +4928,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="18" customHeight="1" s="18">
       <c r="A5" s="26" t="inlineStr">
         <is>
@@ -4914,12 +4939,12 @@
           <t>DD-HSSV-ALL (DD-API-001 -&gt; 006, DD-BAT-001 -&gt; 004)</t>
         </is>
       </c>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="28" t="n"/>
-      <c r="E5" s="28" t="n"/>
-      <c r="F5" s="28" t="n"/>
-      <c r="G5" s="28" t="n"/>
-      <c r="H5" s="28" t="n"/>
+      <c r="C5" s="41" t="n"/>
+      <c r="D5" s="41" t="n"/>
+      <c r="E5" s="41" t="n"/>
+      <c r="F5" s="41" t="n"/>
+      <c r="G5" s="41" t="n"/>
+      <c r="H5" s="42" t="n"/>
       <c r="I5" s="29" t="n"/>
       <c r="J5" s="29" t="n"/>
     </row>
@@ -4934,12 +4959,12 @@
           <t>F-HSSV-001 đến F-HSSV-007, API-HSSV-001 đến API-HSSV-006, SCR-HSSV-001 đến SCR-HSSV-004, BAT-HSSV-001 đến BAT-HSSV-005</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="28" t="n"/>
-      <c r="E6" s="28" t="n"/>
-      <c r="F6" s="28" t="n"/>
-      <c r="G6" s="28" t="n"/>
-      <c r="H6" s="28" t="n"/>
+      <c r="C6" s="41" t="n"/>
+      <c r="D6" s="41" t="n"/>
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="41" t="n"/>
+      <c r="G6" s="41" t="n"/>
+      <c r="H6" s="42" t="n"/>
       <c r="I6" s="29" t="n"/>
       <c r="J6" s="29" t="n"/>
     </row>
@@ -4954,12 +4979,12 @@
           <t>A (Đầy đủ mọi sheet: I/O, Thuật toán chi tiết từng bước, SQL định nghĩa 5 kịch bản, Ma trận Validation, Exception &amp; Log, Unit Test phủ toàn diện)</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="28" t="n"/>
-      <c r="E7" s="28" t="n"/>
-      <c r="F7" s="28" t="n"/>
-      <c r="G7" s="28" t="n"/>
-      <c r="H7" s="28" t="n"/>
+      <c r="C7" s="41" t="n"/>
+      <c r="D7" s="41" t="n"/>
+      <c r="E7" s="41" t="n"/>
+      <c r="F7" s="41" t="n"/>
+      <c r="G7" s="41" t="n"/>
+      <c r="H7" s="42" t="n"/>
       <c r="I7" s="29" t="n"/>
       <c r="J7" s="29" t="n"/>
     </row>
@@ -4977,12 +5002,12 @@
 4. Async Export Worker: Nhận lệnh POST export -&gt; Tạo Job PENDING -&gt; Đẩy vào Redis Queue -&gt; Celery/Spring Worker streaming dữ liệu ra file XLSX/CSV -&gt; Đẩy lên MinIO/S3 -&gt; Trả Presigned Download URL.</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n"/>
-      <c r="D8" s="28" t="n"/>
-      <c r="E8" s="28" t="n"/>
-      <c r="F8" s="28" t="n"/>
-      <c r="G8" s="28" t="n"/>
-      <c r="H8" s="28" t="n"/>
+      <c r="C8" s="41" t="n"/>
+      <c r="D8" s="41" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="41" t="n"/>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="42" t="n"/>
       <c r="I8" s="29" t="n"/>
       <c r="J8" s="29" t="n"/>
     </row>
@@ -5001,12 +5026,12 @@
 DTO: vn.gov.bhxh.hssv.dto.*, Entity: vn.gov.bhxh.hssv.entity.*</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n"/>
-      <c r="D9" s="28" t="n"/>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
-      <c r="H9" s="28" t="n"/>
+      <c r="C9" s="41" t="n"/>
+      <c r="D9" s="41" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="41" t="n"/>
+      <c r="G9" s="41" t="n"/>
+      <c r="H9" s="42" t="n"/>
       <c r="I9" s="29" t="n"/>
       <c r="J9" s="29" t="n"/>
     </row>
@@ -5027,12 +5052,12 @@
 7. void executeMedallionPipeline(PipelineConfig config)</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n"/>
-      <c r="D10" s="28" t="n"/>
-      <c r="E10" s="28" t="n"/>
-      <c r="F10" s="28" t="n"/>
-      <c r="G10" s="28" t="n"/>
-      <c r="H10" s="28" t="n"/>
+      <c r="C10" s="41" t="n"/>
+      <c r="D10" s="41" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="41" t="n"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="42" t="n"/>
       <c r="I10" s="29" t="n"/>
       <c r="J10" s="29" t="n"/>
     </row>
@@ -5047,12 +5072,12 @@
           <t>Clients Web UI, Hệ thống liên thông ngoài, Batch Job Schedulers (Airflow / Spring Batch)</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="28" t="n"/>
-      <c r="E11" s="28" t="n"/>
-      <c r="F11" s="28" t="n"/>
-      <c r="G11" s="28" t="n"/>
-      <c r="H11" s="28" t="n"/>
+      <c r="C11" s="41" t="n"/>
+      <c r="D11" s="41" t="n"/>
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="41" t="n"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="42" t="n"/>
       <c r="I11" s="29" t="n"/>
       <c r="J11" s="29" t="n"/>
     </row>
@@ -5067,12 +5092,12 @@
           <t>PostgreSQL 16, Redis 7.2, DuckDB Engine, MinIO Object Storage, AuditLogService, MessageResolver</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="28" t="n"/>
-      <c r="G12" s="28" t="n"/>
-      <c r="H12" s="28" t="n"/>
+      <c r="C12" s="41" t="n"/>
+      <c r="D12" s="41" t="n"/>
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="41" t="n"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="42" t="n"/>
       <c r="I12" s="29" t="n"/>
       <c r="J12" s="29" t="n"/>
     </row>
@@ -5087,12 +5112,12 @@
           <t>@Transactional(readOnly = true) cho API tra cứu. Ghi Audit log dùng Propagation.REQUIRES_NEW (lỗi audit không ảnh hưởng response). Batch Pipeline thực hiện theo cơ chế Atomic Swap (idempotent, ghi file/partition tạm rồi hoán đổi).</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="28" t="n"/>
-      <c r="F13" s="28" t="n"/>
-      <c r="G13" s="28" t="n"/>
-      <c r="H13" s="28" t="n"/>
+      <c r="C13" s="41" t="n"/>
+      <c r="D13" s="41" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="41" t="n"/>
+      <c r="G13" s="41" t="n"/>
+      <c r="H13" s="42" t="n"/>
       <c r="I13" s="29" t="n"/>
       <c r="J13" s="29" t="n"/>
     </row>
@@ -5107,12 +5132,12 @@
           <t>Online query chỉ đọc (không khóa). Xuất báo cáo dùng Optimistic Lock (@Version trên bảng SYS_EXPORT_JOB). Giới hạn tối đa 5 tác vụ export chạy song song trên mỗi worker node.</t>
         </is>
       </c>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
-      <c r="G14" s="28" t="n"/>
-      <c r="H14" s="28" t="n"/>
+      <c r="C14" s="41" t="n"/>
+      <c r="D14" s="41" t="n"/>
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="41" t="n"/>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="42" t="n"/>
       <c r="I14" s="29" t="n"/>
       <c r="J14" s="29" t="n"/>
     </row>
@@ -5436,9 +5461,9 @@
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="B11:H11"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B10:H10"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B5:H5"/>
   </mergeCells>
@@ -5538,7 +5563,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -6780,7 +6804,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -8586,7 +8609,7 @@
       </c>
       <c r="B53" s="34" t="inlineStr">
         <is>
-          <t>Làm sạch &amp; Khử trùng: Kiểm tra kiểu dữ liệu, loại bỏ trùng khóa, lọc TRANG_THAI = 1. Các bản ghi lỗi TU_NGAY &gt; DEN_NGAY ghi vào thư mục quarantine.</t>
+          <t>Làm sạch &amp; Khử trùng toàn cục (GlobalDedupTracker): Khử trùng ID xuyên suốt 200 chunks; giữ TRANG_THAI IN (0, 1). Với lỗi đảo ngày TU_NGAY &gt; DEN_NGAY: kích hoạt Smart Repair hoán đổi ngày nếu chu kỳ hợp lệ (25..375 ngày) và gắn cờ _FLAG_DATE_SWAPPED = True; dòng lỗi ngoài chu kỳ ghi vào quarantine. Đảm bảo phương trình bảo toàn: Bronze = Silver + Quarantine + Dedup_Global.</t>
         </is>
       </c>
       <c r="C53" s="34" t="inlineStr">
@@ -8623,7 +8646,7 @@
       </c>
       <c r="B54" s="31" t="inlineStr">
         <is>
-          <t>BAT-002 (Xử lý Ý 1): Lọc tập HSSV T10/2024 -&gt; Anti-join với tập có tham gia T08/2026 -&gt; Áp dụng Tie-break chọn thẻ gốc đại diện -&gt; Ghi BC_HSSV_DUNG_THAM_GIA tầng Gold -&gt; Tổng hợp 63 tỉnh.</t>
+          <t>BAT-002 (Xử lý Ý 1): Lọc thẻ hợp lệ TRANG_THAI=1 -&gt; Lọc tập HSSV T10/2024 -&gt; Anti-join với tập có tham gia bất kỳ khối nào tại T08/2026 -&gt; Áp dụng Tie-break (SV &gt; HS, DEN_NGAY DESC, SO_THE_KCB ASC) chọn thẻ gốc đại diện -&gt; Ghi Atomic Rename ra BC_HSSV_DUNG_THAM_GIA tầng Gold -&gt; Tổng hợp 63 tỉnh.</t>
         </is>
       </c>
       <c r="C54" s="27" t="inlineStr">
@@ -8660,7 +8683,7 @@
       </c>
       <c r="B55" s="36" t="inlineStr">
         <is>
-          <t>BAT-003 (Xử lý Ý 2): Lọc người có thẻ T10/2024 (HS/SV) và có thẻ T07/2026 (bất kỳ khối) -&gt; Chạy Window Function và Interval Merging gộp thẻ -&gt; Tính tổng gap_days trong kỳ [2024-10-01, 2026-07-31] -&gt; Lọc gap_days &gt;= 90 -&gt; Ghi BC_HSSV_GIAN_DOAN_BHYT và bảng phân bố.</t>
+          <t>BAT-003 (Xử lý Ý 2): Lọc ứng viên thỏa mãn đồng thời thẻ T10/2024 (HS/SV) và thẻ T07/2026 (bất kỳ khối) -&gt; Cắt biên về kỳ [2024-10-01, 2026-07-31] -&gt; Chạy Window Function MAX(den) OVER (ROWS UNBOUNDED PRECEDING AND 1 PRECEDING) gộp thẻ liên tục/chồng lấn/lồng nhau -&gt; Tính tổng gap_days (cả 2 biên đầu/cuối kỳ và giữa các đoạn) -&gt; Lọc gap_days &gt;= 90 -&gt; Ghi BC_HSSV_GIAN_DOAN_BHYT và bảng phân bố.</t>
         </is>
       </c>
       <c r="C55" s="34" t="inlineStr">
@@ -8916,7 +8939,11 @@
  ORDER BY
    CASE WHEN :sortBy = 'soSoBhxh' AND :sortOrder = 'ASC' THEN P.SO_SO_BHXH END ASC,
    CASE WHEN :sortBy = 'soSoBhxh' AND :sortOrder = 'DESC' THEN P.SO_SO_BHXH END DESC,
-   CASE WHEN :sortBy = 'soNgayGianDoan' AND :sortOrder = 'DESC' THEN P.SO_NGAY_GIAN_DOAN END DESC
+   CASE WHEN :sortBy = 'hoTen' AND :sortOrder = 'ASC' THEN P.HO_TEN END ASC,
+   CASE WHEN :sortBy = 'hoTen' AND :sortOrder = 'DESC' THEN P.HO_TEN END DESC,
+   CASE WHEN :sortBy = 'soNgayGianDoan' AND :sortOrder = 'ASC' THEN P.SO_NGAY_GIAN_DOAN END ASC,
+   CASE WHEN :sortBy = 'soNgayGianDoan' AND :sortOrder = 'DESC' THEN P.SO_NGAY_GIAN_DOAN END DESC,
+   P.SO_SO_BHXH ASC
  LIMIT :pageSize OFFSET :offset;</t>
         </is>
       </c>
@@ -9172,8 +9199,12 @@
   FROM TK_DBHC_HSSV_TONG_HOP T
  ORDER BY
    CASE WHEN :sortBy = 'maTinh' AND :sortOrder = 'ASC' THEN T.MA_TINH END ASC,
+   CASE WHEN :sortBy = 'maTinh' AND :sortOrder = 'DESC' THEN T.MA_TINH END DESC,
+   CASE WHEN :sortBy = 'tongDung' AND :sortOrder = 'ASC' THEN T.TONG_SO_DUNG END ASC,
    CASE WHEN :sortBy = 'tongDung' AND :sortOrder = 'DESC' THEN T.TONG_SO_DUNG END DESC,
-   CASE WHEN :sortBy = 'tongGianDoan' AND :sortOrder = 'DESC' THEN T.TONG_SO_GIAN_DOAN END DESC;</t>
+   CASE WHEN :sortBy = 'tongGianDoan' AND :sortOrder = 'ASC' THEN T.TONG_SO_GIAN_DOAN END ASC,
+   CASE WHEN :sortBy = 'tongGianDoan' AND :sortOrder = 'DESC' THEN T.TONG_SO_GIAN_DOAN END DESC,
+   T.MA_TINH ASC;</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
@@ -9363,38 +9394,79 @@
       </c>
       <c r="C13" s="39" t="inlineStr">
         <is>
-          <t>-- Tầng xử lý DuckDB SQL trên 200M dòng thẻ BHYT
-WITH base_cards AS (
-    SELECT SO_SO_BHXH, TU_NGAY, DEN_NGAY,
-           LAG(DEN_NGAY) OVER (PARTITION BY SO_SO_BHXH ORDER BY TU_NGAY, DEN_NGAY) AS PREV_DEN_NGAY
+          <t>-- Tầng xử lý DuckDB SQL trên 200M dòng thẻ BHYT (Chuẩn hóa theo gold_logic_y2.py Tuần 2)
+WITH valid_cards AS (
+    SELECT SO_SO_BHXH, MA_KHOI, TU_NGAY, DEN_NGAY,
+           GREATEST(TU_NGAY, DATE '2024-10-01') AS tu_clip,
+           LEAST(DEN_NGAY, DATE '2026-07-31') AS den_clip
       FROM st_inthe_dtl_silver
      WHERE TRANG_THAI = 1
-       AND TU_NGAY &lt;= DATE '2026-07-31'
-       AND DEN_NGAY &gt;= DATE '2024-10-01'
+),
+candidates AS (
+    -- Thỏa mãn đồng thời ĐK1 (HSSV tại T10/2024) và ĐK2 (còn tham gia bất kỳ khối tại T07/2026)
+    SELECT DISTINCT b.SO_SO_BHXH
+      FROM valid_cards b
+      JOIN valid_cards c ON b.SO_SO_BHXH = c.SO_SO_BHXH
+     WHERE b.MA_KHOI IN ('HS', 'SV')
+       AND b.TU_NGAY &lt; DATE '2024-11-01' AND b.DEN_NGAY &gt;= DATE '2024-10-01'
+       AND c.TU_NGAY &lt; DATE '2026-08-01' AND c.DEN_NGAY &gt;= DATE '2026-07-01'
+),
+cand_window_cards AS (
+    SELECT v.SO_SO_BHXH, v.tu_clip AS tu, v.den_clip AS den
+      FROM valid_cards v
+      JOIN candidates cd ON v.SO_SO_BHXH = cd.SO_SO_BHXH
+     WHERE v.tu_clip &lt;= v.den_clip
+),
+with_prev AS (
+    -- Dùng MAX(den) OVER (... UNBOUNDED PRECEDING AND 1 PRECEDING) xử lý triệt để thẻ lồng nhau
+    SELECT SO_SO_BHXH, tu, den,
+           MAX(den) OVER (
+               PARTITION BY SO_SO_BHXH ORDER BY tu, den
+               ROWS BETWEEN UNBOUNDED PRECEDING AND 1 PRECEDING
+           ) AS prev_max_den
+      FROM cand_window_cards
 ),
 marked_islands AS (
-    SELECT SO_SO_BHXH, TU_NGAY, DEN_NGAY,
-           CASE WHEN PREV_DEN_NGAY IS NULL OR TU_NGAY &gt; PREV_DEN_NGAY + 1 THEN 1 ELSE 0 END AS IS_NEW_ISLAND
-      FROM base_cards
+    SELECT SO_SO_BHXH, tu, den,
+           CASE WHEN prev_max_den IS NULL OR tu &gt; prev_max_den + INTERVAL 1 DAY THEN 1 ELSE 0 END AS is_new_grp
+      FROM with_prev
 ),
 grouped_islands AS (
-    SELECT SO_SO_BHXH, TU_NGAY, DEN_NGAY,
-           SUM(IS_NEW_ISLAND) OVER (PARTITION BY SO_SO_BHXH ORDER BY TU_NGAY, DEN_NGAY) AS ISLAND_ID
+    SELECT SO_SO_BHXH, tu, den,
+           SUM(is_new_grp) OVER (
+               PARTITION BY SO_SO_BHXH ORDER BY tu, den
+               ROWS UNBOUNDED PRECEDING
+           ) AS grp_id
       FROM marked_islands
 ),
 merged_intervals AS (
-    SELECT SO_SO_BHXH,
-           MIN(TU_NGAY) AS INTERVAL_START,
-           MAX(DEN_NGAY) AS INTERVAL_END
+    SELECT SO_SO_BHXH, grp_id,
+           MIN(tu) AS m_tu,
+           MAX(den) AS m_den
       FROM grouped_islands
-     GROUP BY SO_SO_BHXH, ISLAND_ID
+     GROUP BY SO_SO_BHXH, grp_id
+),
+with_gaps AS (
+    SELECT SO_SO_BHXH, m_tu, m_den,
+           (m_tu - LAG(m_den) OVER (PARTITION BY SO_SO_BHXH ORDER BY m_tu) - 1) AS gap_days
+      FROM merged_intervals
+),
+gap_events AS (
+    SELECT SO_SO_BHXH, gap_days FROM with_gaps WHERE gap_days &gt; 0
+    UNION ALL
+    SELECT SO_SO_BHXH, (MIN(m_tu) - DATE '2024-10-01') AS gap_days
+      FROM merged_intervals GROUP BY SO_SO_BHXH HAVING MIN(m_tu) &gt; DATE '2024-10-01'
+    UNION ALL
+    SELECT SO_SO_BHXH, (DATE '2026-07-31' - MAX(m_den)) AS gap_days
+      FROM merged_intervals GROUP BY SO_SO_BHXH HAVING MAX(m_den) &lt; DATE '2026-07-31'
 )
 SELECT SO_SO_BHXH,
-       COUNT(*) AS SO_KHOANG_LIEN_TUC,
-       -- Tính tổng số ngày gián đoạn trong kỳ xét [2024-10-01, 2026-07-31] (669 ngày)
-       669 - SUM(DATEDIFF('day', GREATEST(INTERVAL_START, DATE '2024-10-01'), LEAST(INTERVAL_END, DATE '2026-07-31')) + 1) AS TONG_NGAY_GIAN_DOAN
-  FROM merged_intervals
- GROUP BY SO_SO_BHXH;</t>
+       COUNT(gap_days) AS SO_DOT_GIAN_DOAN,
+       COALESCE(SUM(gap_days), 0) AS TONG_NGAY_GIAN_DOAN,
+       ROUND(COALESCE(SUM(gap_days), 0) / 30.0, 1) AS SO_THANG_GIAN_DOAN
+  FROM gap_events
+ GROUP BY SO_SO_BHXH
+HAVING COALESCE(SUM(gap_days), 0) &gt;= 90;</t>
         </is>
       </c>
       <c r="D13" s="34" t="inlineStr">
@@ -9409,7 +9481,7 @@
       </c>
       <c r="F13" s="36" t="inlineStr">
         <is>
-          <t>~5.000.000 người HSSV</t>
+          <t>~241.869 người HSSV gián đoạn &gt;= 90 ngày (từ ~5M HSSV)</t>
         </is>
       </c>
       <c r="G13" s="34" t="inlineStr">
@@ -9759,7 +9831,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -10340,12 +10411,12 @@
       </c>
       <c r="D19" s="34" t="inlineStr">
         <is>
-          <t>TU_NGAY &gt; DEN_NGAY</t>
+          <t>TU_NGAY &gt; DEN_NGAY (Xét chu kỳ Δ = TU_NGAY - DEN_NGAY)</t>
         </is>
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>Ghi vào quarantine</t>
+          <t>Nếu 25 &lt;= Δ &lt;= 375d: Smart Repair hoán đổi ngày &amp; gắn _FLAG_DATE_SWAPPED=True; ngược lại ghi vào quarantine</t>
         </is>
       </c>
       <c r="F19" s="35" t="n">
@@ -10702,7 +10773,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="18">
       <c r="A5" s="30" t="inlineStr">
         <is>

</xml_diff>